<commit_message>
Deploying to main from @ set-soft/kibot_variants_arduprog_test@1e1f73bc0b1e218d2ab85a3f36532a25ee384d8b 🚀
</commit_message>
<xml_diff>
--- a/BoM/Costs/t1-bom.xlsx
+++ b/BoM/Costs/t1-bom.xlsx
@@ -589,7 +589,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>9.0.6+1</t>
+    <t>9.0.7+1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -805,10 +805,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2025-11-26 13:17:26</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-05-12 09:34:38</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
   </si>
   <si>
     <t>Resettable fuse, polymeric positive temperature coefficient</t>

</xml_diff>

<commit_message>
Deploying to main from @ set-soft/kibot_variants_arduprog_test@135d77b440a929b8dc4f6d317a81e03ec03b4d04 🚀
</commit_message>
<xml_diff>
--- a/BoM/Costs/t1-bom.xlsx
+++ b/BoM/Costs/t1-bom.xlsx
@@ -290,7 +290,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="193">
   <si>
     <t>Row</t>
   </si>
@@ -367,9 +367,6 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>~</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -589,7 +586,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>9.0.7+1</t>
+    <t>10.0.1-10.0.1~ubuntu25.10.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -805,10 +802,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-05-12 09:34:38</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.6</t>
+    <t>2026-06-03 09:31:45</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.20 + KiBot v1.9.1</t>
   </si>
   <si>
     <t>Resettable fuse, polymeric positive temperature coefficient</t>
@@ -1709,7 +1706,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
     <col min="5" max="5" width="29.7109375" customWidth="1"/>
     <col min="6" max="6" width="46.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
@@ -1727,7 +1724,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -1746,13 +1743,13 @@
     </row>
     <row r="2" spans="1:17">
       <c r="C2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F2" s="3">
         <v>22</v>
@@ -1760,41 +1757,41 @@
     </row>
     <row r="3" spans="1:17">
       <c r="C3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="E3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="C4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="E4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="C5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>97</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -1802,13 +1799,13 @@
     </row>
     <row r="6" spans="1:17">
       <c r="C6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F6" s="3">
         <v>19</v>
@@ -1893,7 +1890,7 @@
         <v>24</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>18</v>
@@ -1922,7 +1919,7 @@
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>18</v>
@@ -1931,10 +1928,10 @@
         <v>19</v>
       </c>
       <c r="D10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>28</v>
       </c>
       <c r="F10" s="10" t="s">
         <v>22</v>
@@ -1946,7 +1943,7 @@
         <v>24</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>18</v>
@@ -1975,22 +1972,22 @@
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="E11" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="7" t="s">
         <v>32</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>33</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>17</v>
@@ -1999,16 +1996,16 @@
         <v>24</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="K11" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="L11" s="11" t="s">
         <v>34</v>
-      </c>
-      <c r="L11" s="11" t="s">
-        <v>35</v>
       </c>
       <c r="M11" s="6" t="s">
         <v>18</v>
@@ -2034,16 +2031,16 @@
         <v>18</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>38</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>39</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>17</v>
@@ -2052,7 +2049,7 @@
         <v>24</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>18</v>
@@ -2067,10 +2064,10 @@
         <v>18</v>
       </c>
       <c r="N12" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O12" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P12" s="9" t="s">
         <v>18</v>
@@ -2081,40 +2078,40 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="D13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>44</v>
-      </c>
       <c r="G13" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>24</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>18</v>
       </c>
       <c r="K13" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="L13" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>46</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>18</v>
@@ -2134,22 +2131,22 @@
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>49</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="F14" s="10" t="s">
-        <v>50</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>17</v>
@@ -2158,16 +2155,16 @@
         <v>24</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>18</v>
       </c>
       <c r="K14" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="L14" s="12" t="s">
         <v>51</v>
-      </c>
-      <c r="L14" s="12" t="s">
-        <v>52</v>
       </c>
       <c r="M14" s="9" t="s">
         <v>18</v>
@@ -2187,22 +2184,22 @@
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="7" t="s">
+      <c r="D15" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>17</v>
@@ -2211,16 +2208,16 @@
         <v>24</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J15" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="K15" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="K15" s="11" t="s">
+      <c r="L15" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="M15" s="6" t="s">
         <v>18</v>
@@ -2240,22 +2237,22 @@
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>64</v>
-      </c>
-      <c r="F16" s="10" t="s">
-        <v>65</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>17</v>
@@ -2264,7 +2261,7 @@
         <v>24</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J16" s="9" t="s">
         <v>18</v>
@@ -2293,22 +2290,22 @@
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="7" t="s">
+      <c r="D17" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>70</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>17</v>
@@ -2317,7 +2314,7 @@
         <v>24</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>18</v>
@@ -2346,22 +2343,22 @@
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="B18" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="E18" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>73</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>74</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>17</v>
@@ -2370,7 +2367,7 @@
         <v>24</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J18" s="9" t="s">
         <v>18</v>
@@ -2399,31 +2396,31 @@
     </row>
     <row r="19" spans="1:17">
       <c r="A19" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="7" t="s">
+      <c r="D19" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="E19" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="F19" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>79</v>
-      </c>
       <c r="G19" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>24</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>18</v>
@@ -2452,22 +2449,22 @@
     </row>
     <row r="20" spans="1:17">
       <c r="A20" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D20" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="10" t="s">
+      <c r="E20" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="10" t="s">
-        <v>82</v>
-      </c>
       <c r="F20" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>17</v>
@@ -2476,7 +2473,7 @@
         <v>24</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J20" s="9" t="s">
         <v>18</v>
@@ -2505,22 +2502,22 @@
     </row>
     <row r="21" spans="1:17">
       <c r="A21" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>17</v>
@@ -2529,7 +2526,7 @@
         <v>24</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J21" s="6" t="s">
         <v>18</v>
@@ -2574,7 +2571,7 @@
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="27.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="44.7109375" customWidth="1"/>
     <col min="7" max="7" width="26.7109375" customWidth="1"/>
@@ -2592,7 +2589,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -2611,13 +2608,13 @@
     </row>
     <row r="2" spans="1:17">
       <c r="C2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="E2" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F2" s="3">
         <v>22</v>
@@ -2625,41 +2622,41 @@
     </row>
     <row r="3" spans="1:17">
       <c r="C3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="E3" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="C4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="E4" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="C5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>97</v>
-      </c>
       <c r="E5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -2667,13 +2664,13 @@
     </row>
     <row r="6" spans="1:17">
       <c r="C6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>99</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F6" s="3">
         <v>19</v>
@@ -2743,25 +2740,25 @@
         <v>19</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>108</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>22</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H9" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>110</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>18</v>
@@ -2787,34 +2784,34 @@
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="E10" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>113</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>17</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K10" s="9" t="s">
         <v>18</v>
@@ -2840,40 +2837,40 @@
     </row>
     <row r="11" spans="1:17">
       <c r="A11" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="E11" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>118</v>
-      </c>
       <c r="F11" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J11" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M11" s="6" t="s">
         <v>18</v>
@@ -2899,34 +2896,34 @@
         <v>18</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="E12" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="F12" s="10" t="s">
         <v>122</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>123</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>17</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J12" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="K12" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="L12" s="12" t="s">
         <v>124</v>
-      </c>
-      <c r="K12" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="L12" s="12" t="s">
-        <v>125</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>18</v>
@@ -2946,40 +2943,40 @@
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="E13" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>127</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>128</v>
       </c>
       <c r="G13" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J13" s="11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K13" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="L13" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>130</v>
       </c>
       <c r="M13" s="6" t="s">
         <v>18</v>
@@ -2999,34 +2996,34 @@
     </row>
     <row r="14" spans="1:17">
       <c r="A14" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B14" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D14" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="E14" s="10" t="s">
-        <v>132</v>
-      </c>
       <c r="F14" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K14" s="9" t="s">
         <v>18</v>
@@ -3052,34 +3049,34 @@
     </row>
     <row r="15" spans="1:17">
       <c r="A15" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D15" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="E15" s="7" t="s">
-        <v>134</v>
-      </c>
       <c r="F15" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G15" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H15" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>110</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>18</v>
@@ -3105,93 +3102,93 @@
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B16" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="E16" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="G16" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="K16" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="I16" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="K16" s="12" t="s">
+      <c r="L16" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="M16" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="L16" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="M16" s="12" t="s">
+      <c r="N16" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="N16" s="12" t="s">
+      <c r="O16" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="O16" s="12" t="s">
+      <c r="P16" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="P16" s="12" t="s">
+      <c r="Q16" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="Q16" s="12" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="17" spans="1:17">
       <c r="A17" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C17" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="7" t="s">
         <v>147</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>148</v>
       </c>
       <c r="G17" s="5" t="s">
         <v>17</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J17" s="11" t="s">
-        <v>110</v>
-      </c>
       <c r="K17" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="L17" s="11" t="s">
         <v>149</v>
-      </c>
-      <c r="L17" s="11" t="s">
-        <v>150</v>
       </c>
       <c r="M17" s="6" t="s">
         <v>18</v>
@@ -3236,7 +3233,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -3245,13 +3242,13 @@
     </row>
     <row r="2" spans="1:8">
       <c r="D2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="G2" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -3259,13 +3256,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="D3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="G3" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -3274,13 +3271,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="D4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="G4" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H22)</f>
@@ -3289,23 +3286,23 @@
     </row>
     <row r="5" spans="1:8">
       <c r="D5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -3329,16 +3326,16 @@
         <v>5</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="18" t="s">
         <v>154</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -3349,7 +3346,7 @@
         <v>21</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>22</v>
@@ -3365,13 +3362,13 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>28</v>
-      </c>
       <c r="C11" s="19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D11" s="19" t="s">
         <v>22</v>
@@ -3387,16 +3384,16 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="C12" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>32</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>33</v>
       </c>
       <c r="F12" s="19">
         <f>BoardQty*1</f>
@@ -3409,16 +3406,16 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="C13" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" s="19" t="s">
         <v>38</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>39</v>
       </c>
       <c r="F13" s="19">
         <f>BoardQty*1</f>
@@ -3431,16 +3428,16 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>43</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>44</v>
       </c>
       <c r="F14" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -3453,16 +3450,16 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="D15" s="19" t="s">
         <v>49</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="D15" s="19" t="s">
-        <v>50</v>
       </c>
       <c r="F15" s="19">
         <f>BoardQty*1</f>
@@ -3475,16 +3472,16 @@
     </row>
     <row r="16" spans="1:8" ht="45" customHeight="1">
       <c r="A16" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="C16" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="D16" s="19" t="s">
         <v>56</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="D16" s="19" t="s">
-        <v>57</v>
       </c>
       <c r="F16" s="19">
         <f>BoardQty*1</f>
@@ -3497,16 +3494,16 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="C17" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="19" t="s">
         <v>64</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>65</v>
       </c>
       <c r="F17" s="19">
         <f>BoardQty*1</f>
@@ -3519,16 +3516,16 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="C18" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" s="19" t="s">
         <v>69</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>70</v>
       </c>
       <c r="F18" s="19">
         <f>BoardQty*1</f>
@@ -3541,16 +3538,16 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" s="19" t="s">
         <v>73</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>74</v>
       </c>
       <c r="F19" s="19">
         <f>BoardQty*1</f>
@@ -3563,16 +3560,16 @@
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="C20" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="D20" s="19" t="s">
         <v>78</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="D20" s="19" t="s">
-        <v>79</v>
       </c>
       <c r="F20" s="19">
         <f>CEILING(BoardQty*3,1)</f>
@@ -3585,16 +3582,16 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B21" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="19" t="s">
-        <v>82</v>
-      </c>
       <c r="C21" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F21" s="19">
         <f>BoardQty*1</f>
@@ -3607,19 +3604,19 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="C22" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D22" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="D22" s="19" t="s">
+      <c r="E22" s="19" t="s">
         <v>87</v>
-      </c>
-      <c r="E22" s="19" t="s">
-        <v>88</v>
       </c>
       <c r="F22" s="19">
         <f>BoardQty*1</f>
@@ -3632,15 +3629,15 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="B25" s="22" t="s">
         <v>170</v>
-      </c>
-      <c r="B25" s="22" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3731,7 +3728,7 @@
     <col min="2" max="2" width="15.7109375" customWidth="1"/>
     <col min="3" max="3" width="61.7109375" customWidth="1" outlineLevel="2"/>
     <col min="4" max="4" width="40.7109375" customWidth="1" outlineLevel="2"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="28.7109375" customWidth="1" outlineLevel="1"/>
     <col min="6" max="6" width="17.7109375" customWidth="1" outlineLevel="1"/>
     <col min="7" max="7" width="15.7109375" customWidth="1"/>
     <col min="8" max="8" width="16.7109375" customWidth="1"/>
@@ -3739,7 +3736,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1">
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
@@ -3748,13 +3745,13 @@
     </row>
     <row r="2" spans="1:8">
       <c r="D2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>91</v>
-      </c>
       <c r="G2" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H2" s="13">
         <v>1</v>
@@ -3762,13 +3759,13 @@
     </row>
     <row r="3" spans="1:8">
       <c r="D3" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="G3" s="14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H3" s="15">
         <f>TotalCost/BoardQty</f>
@@ -3777,13 +3774,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="D4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="G4" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H4" s="16">
         <f>SUM(H10:H18)</f>
@@ -3792,23 +3789,23 @@
     </row>
     <row r="5" spans="1:8">
       <c r="D5" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="D6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="17" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -3832,27 +3829,27 @@
         <v>5</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="18" t="s">
         <v>154</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="19" t="s">
-        <v>108</v>
-      </c>
       <c r="C10" s="19" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>22</v>
@@ -3868,16 +3865,16 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="C11" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>113</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>114</v>
       </c>
       <c r="F11" s="19">
         <f>BoardQty*1</f>
@@ -3890,16 +3887,16 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="19" t="s">
         <v>117</v>
       </c>
-      <c r="B12" s="19" t="s">
-        <v>118</v>
-      </c>
       <c r="C12" s="19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F12" s="19">
         <f>BoardQty*1</f>
@@ -3912,16 +3909,16 @@
     </row>
     <row r="13" spans="1:8" ht="45" customHeight="1">
       <c r="A13" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="C13" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="D13" s="19" t="s">
         <v>122</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>123</v>
       </c>
       <c r="F13" s="19">
         <f>BoardQty*1</f>
@@ -3934,16 +3931,16 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>127</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>126</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>128</v>
       </c>
       <c r="F14" s="19">
         <f>BoardQty*1</f>
@@ -3956,16 +3953,16 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="B15" s="19" t="s">
-        <v>132</v>
-      </c>
       <c r="C15" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F15" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -3978,16 +3975,16 @@
     </row>
     <row r="16" spans="1:8">
       <c r="A16" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>134</v>
-      </c>
       <c r="C16" s="19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F16" s="19">
         <f>BoardQty*1</f>
@@ -4000,16 +3997,16 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="19" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="C17" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="D17" s="19" t="s">
         <v>137</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>138</v>
       </c>
       <c r="F17" s="19">
         <f>CEILING(BoardQty*2,1)</f>
@@ -4022,16 +4019,16 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="C18" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="D18" s="19" t="s">
         <v>147</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>178</v>
-      </c>
-      <c r="D18" s="19" t="s">
-        <v>148</v>
       </c>
       <c r="F18" s="19">
         <f>BoardQty*1</f>
@@ -4044,15 +4041,15 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="B21" s="22" t="s">
         <v>170</v>
-      </c>
-      <c r="B21" s="22" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:8">
       <c r="A22" s="23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -4121,77 +4118,77 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="24" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="25" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="26" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="28" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="29" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="30" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="32" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>